<commit_message>
Aggiornamento dati con test_bis.xlsx: nomi completi e 14 Professional Avezzano - Sostituito test.xlsx con test_bis.xlsx contenente nomi completi - Dirigente Milano: 25, Professional Milano: 17, Dirigente Avezzano: 7, Professional Avezzano: 14 - Rigenerati tutti i grafici (barchart, heatmap, radar chart, classifiche) - Aggiunti radar chart individuali con nomi completi
Co-authored-by: spastoris <spastoris@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/analisi_competenze.xlsx
+++ b/analisi_competenze.xlsx
@@ -499,7 +499,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Dir Milano 1</t>
+          <t>Batavia Marco Filippo</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -550,7 +550,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Dir Milano 2</t>
+          <t>Moraja Marco</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -601,7 +601,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Dir Milano 3</t>
+          <t>Gallina Paolo</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -652,7 +652,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Dir Milano 4</t>
+          <t>Zilio Stefano</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -703,7 +703,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Dir Milano 5</t>
+          <t>Campestri Ilaria</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -754,7 +754,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Dir Milano 6</t>
+          <t>Gerevini Mara Bianca</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -805,7 +805,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Dir Milano 7</t>
+          <t>Fumagalli Luca</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -856,7 +856,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Dir Milano 8</t>
+          <t>Riva Mauro</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -907,7 +907,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Dir Milano 9</t>
+          <t>Giorgi Stefano</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -958,7 +958,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Dir Milano 10</t>
+          <t>Foglia Emanuela</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1009,7 +1009,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Dir Milano 11</t>
+          <t>Alacqua Stefano</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1060,7 +1060,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Dir Milano 12</t>
+          <t>Mura Michele</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1111,7 +1111,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Dir Milano 13</t>
+          <t>Gallino federico</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1162,7 +1162,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Dir Milano 14</t>
+          <t>Rondena Segio</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1213,7 +1213,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Dir Milano 15</t>
+          <t>Zucchi Imerio</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1264,7 +1264,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Dir Milano 16</t>
+          <t>Nicolosi Dario</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1315,7 +1315,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Dir Milano 17</t>
+          <t>Mio Bertolo Johnny</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1366,7 +1366,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Dir Milano 18</t>
+          <t xml:space="preserve">Battilana Paolo </t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1417,7 +1417,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Dir Milano 19</t>
+          <t>Vergani Giorgio</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1468,7 +1468,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Dir Milano 20</t>
+          <t>Maccalini Enrico</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1519,7 +1519,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Dir Milano 21</t>
+          <t>Vacca Paolo</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1570,7 +1570,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Dir Milano 22</t>
+          <t>Gigli Jabril</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1621,7 +1621,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Dir Milano 23</t>
+          <t>Tradani Susanna</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1672,7 +1672,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Dir Milano 24</t>
+          <t>Cadoppi Andrea</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1723,7 +1723,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Dir Milano 25</t>
+          <t>Valcamonica Marco</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1774,7 +1774,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Pro Milano 1</t>
+          <t>Muca Adrian</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1825,7 +1825,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Pro Milano 2</t>
+          <t>Farina Simona</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1876,7 +1876,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Pro Milano 3</t>
+          <t>Fumagalli Alessandro</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1927,7 +1927,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Pro Milano 4</t>
+          <t>Arco Carmelo</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1978,7 +1978,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Pro Milano 5</t>
+          <t>Macchi Giorgio</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2029,7 +2029,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Pro Milano 6</t>
+          <t>Premoli Gianluca</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2080,7 +2080,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Pro Milano 7</t>
+          <t>Colombo A lessandra</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2131,7 +2131,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Pro Milano 8</t>
+          <t>Fernicola Alessandra</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2182,7 +2182,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Pro Milano 9</t>
+          <t>Toia Luca Luigi</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2233,7 +2233,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Pro Milano 10</t>
+          <t>Campanello Marco</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2284,7 +2284,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Pro Milano 11</t>
+          <t>Milanta Mariapaola</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2335,7 +2335,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Pro Milano 12</t>
+          <t>Calderoni Gabriele Maria</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2386,7 +2386,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Pro Milano 13</t>
+          <t>Ceriani Massimo</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2437,7 +2437,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Pro Milano 14</t>
+          <t>Valieri Andrea</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2488,7 +2488,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Pro Milano 15</t>
+          <t>Mauri Luca</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2539,7 +2539,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Pro Milano 16</t>
+          <t>Cercaci Alessandra</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2590,7 +2590,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Pro Milano 17</t>
+          <t>Roberto Rocca</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2641,7 +2641,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Dir Avezzano 1</t>
+          <t>Di Sabatino Bruno</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2692,7 +2692,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Dir Avezzano 2</t>
+          <t xml:space="preserve">Diego Gi Giampietro </t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2743,7 +2743,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Dir Avezzano 3</t>
+          <t>Francesconi Luigia</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2794,7 +2794,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Dir Avezzano 4</t>
+          <t>Properzi Massimiliano</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2845,7 +2845,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Dir Avezzano 5</t>
+          <t>Santangelo Maurizio</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2896,7 +2896,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Dir Avezzano 6</t>
+          <t>Santella Gianni</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2947,7 +2947,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Dir Avezzano 7</t>
+          <t>Tartaglia Vincenzo</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2998,7 +2998,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Pro Avezzano 1</t>
+          <t xml:space="preserve">Bianchi Liberato </t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3049,12 +3049,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Pro Avezzano 2</t>
+          <t xml:space="preserve">Castrigano Luca </t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Dirigente Avezzano</t>
+          <t>Professional Avezzano</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -3100,12 +3100,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Pro Avezzano 3</t>
+          <t xml:space="preserve">De Amicis Alvaro </t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Dirigente Avezzano</t>
+          <t>Professional Avezzano</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -3151,12 +3151,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Pro Avezzano 4</t>
+          <t xml:space="preserve">Di Giacomo Lorenzo </t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Dirigente Avezzano</t>
+          <t>Professional Avezzano</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -3202,12 +3202,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Pro Avezzano 5</t>
+          <t>Di Paolo Massimo</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Dirigente Avezzano</t>
+          <t>Professional Avezzano</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -3253,12 +3253,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Pro Avezzano 6</t>
+          <t xml:space="preserve">Volpa Alessandra </t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Dirigente Avezzano</t>
+          <t>Professional Avezzano</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -3304,12 +3304,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Pro Avezzano 7</t>
+          <t>Amabrini Fabio</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Dirigente Avezzano</t>
+          <t>Professional Avezzano</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -3355,12 +3355,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Pro Avezzano 8</t>
+          <t>Ghidelli Serge</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Dirigente Avezzano</t>
+          <t>Professional Avezzano</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -3406,12 +3406,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Pro Avezzano 9</t>
+          <t>Margutti Pasquale</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Dirigente Avezzano</t>
+          <t>Professional Avezzano</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -3457,12 +3457,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Pro Avezzano 10</t>
+          <t>Palma Luca</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Dirigente Avezzano</t>
+          <t>Professional Avezzano</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -3508,12 +3508,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Pro Avezzano 11</t>
+          <t>Piccirilli Gianluca</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Dirigente Avezzano</t>
+          <t>Professional Avezzano</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -3559,12 +3559,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Pro Avezzano 12</t>
+          <t>Tellone Giuliano</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Dirigente Avezzano</t>
+          <t>Professional Avezzano</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -3610,12 +3610,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Pro Avezzano 13</t>
+          <t>Zaccardelli Giuseppe</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Dirigente Avezzano</t>
+          <t>Professional Avezzano</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -3661,12 +3661,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Pro Avezzano 14</t>
+          <t>Lamura Sabrina</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Dirigente Avezzano</t>
+          <t>Professional Avezzano</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -4266,40 +4266,40 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3.25</v>
+        <v>3.142857142857143</v>
       </c>
       <c r="C2" t="n">
-        <v>2.775</v>
+        <v>2.642857142857143</v>
       </c>
       <c r="D2" t="n">
-        <v>2.925</v>
+        <v>2.928571428571428</v>
       </c>
       <c r="E2" t="n">
-        <v>2.975</v>
+        <v>3.142857142857143</v>
       </c>
       <c r="F2" t="n">
-        <v>2.725</v>
+        <v>2.571428571428572</v>
       </c>
       <c r="G2" t="n">
-        <v>2.75</v>
+        <v>2.571428571428572</v>
       </c>
       <c r="H2" t="n">
-        <v>3.075</v>
+        <v>3.214285714285714</v>
       </c>
       <c r="I2" t="n">
-        <v>2.9</v>
+        <v>3.071428571428572</v>
       </c>
       <c r="J2" t="n">
-        <v>2.525</v>
+        <v>2.642857142857143</v>
       </c>
       <c r="K2" t="n">
-        <v>2.7</v>
+        <v>2.857142857142857</v>
       </c>
       <c r="L2" t="n">
-        <v>2.925</v>
+        <v>2.857142857142857</v>
       </c>
       <c r="M2" t="n">
-        <v>2.75</v>
+        <v>2.857142857142857</v>
       </c>
     </row>
     <row r="3">
@@ -4352,40 +4352,40 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3.5</v>
+        <v>3.321428571428572</v>
       </c>
       <c r="C4" t="n">
-        <v>3.5</v>
+        <v>2.892857142857143</v>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>2.928571428571428</v>
       </c>
       <c r="E4" t="n">
-        <v>3</v>
+        <v>2.892857142857143</v>
       </c>
       <c r="F4" t="n">
-        <v>2.5</v>
+        <v>2.785714285714286</v>
       </c>
       <c r="G4" t="n">
-        <v>3</v>
+        <v>2.857142857142857</v>
       </c>
       <c r="H4" t="n">
         <v>3</v>
       </c>
       <c r="I4" t="n">
-        <v>3.5</v>
+        <v>2.857142857142857</v>
       </c>
       <c r="J4" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="K4" t="n">
-        <v>2.5</v>
+        <v>2.607142857142857</v>
       </c>
       <c r="L4" t="n">
-        <v>3</v>
+        <v>2.964285714285714</v>
       </c>
       <c r="M4" t="n">
-        <v>2</v>
+        <v>2.642857142857143</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Rigenerazione dati con test_tris.xlsx - 66 individui (26 Dirigente Milano, 17 Professional Milano, 7 Dirigente Avezzano, 16 Professional Avezzano)
Co-authored-by: spastoris <spastoris@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/analisi_competenze.xlsx
+++ b/analisi_competenze.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O64"/>
+  <dimension ref="A1:O67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1774,40 +1774,40 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Muca Adrian</t>
+          <t>De cesaro Franco</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Professional Milano</t>
+          <t>Dirigente Milano</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="D27" t="n">
         <v>2.5</v>
       </c>
       <c r="E27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F27" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="G27" t="n">
-        <v>2</v>
+        <v>3.5</v>
       </c>
       <c r="H27" t="n">
         <v>3</v>
       </c>
       <c r="I27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J27" t="n">
         <v>3</v>
       </c>
       <c r="K27" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="L27" t="n">
         <v>2.5</v>
@@ -1819,13 +1819,13 @@
         <v>2.5</v>
       </c>
       <c r="O27" t="n">
-        <v>2.958333333333333</v>
+        <v>2.79</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Farina Simona</t>
+          <t>Muca Adrian</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1846,37 +1846,37 @@
         <v>3</v>
       </c>
       <c r="G28" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="H28" t="n">
         <v>3</v>
       </c>
       <c r="I28" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J28" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="K28" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="L28" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="M28" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="N28" t="n">
         <v>2.5</v>
       </c>
       <c r="O28" t="n">
-        <v>2.791666666666667</v>
+        <v>2.958333333333333</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Fumagalli Alessandro</t>
+          <t>Farina Simona</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1885,7 +1885,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="D29" t="n">
         <v>2.5</v>
@@ -1897,37 +1897,37 @@
         <v>3</v>
       </c>
       <c r="G29" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="H29" t="n">
         <v>3</v>
       </c>
       <c r="I29" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="J29" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="K29" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="L29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M29" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="N29" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="O29" t="n">
-        <v>2.958333333333333</v>
+        <v>2.791666666666667</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Arco Carmelo</t>
+          <t>Fumagalli Alessandro</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1936,19 +1936,19 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="D30" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="E30" t="n">
         <v>3</v>
       </c>
       <c r="F30" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="G30" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="H30" t="n">
         <v>3</v>
@@ -1957,7 +1957,7 @@
         <v>3.5</v>
       </c>
       <c r="J30" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="K30" t="n">
         <v>3</v>
@@ -1966,19 +1966,19 @@
         <v>3</v>
       </c>
       <c r="M30" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="N30" t="n">
         <v>3</v>
       </c>
       <c r="O30" t="n">
-        <v>3.125</v>
+        <v>2.958333333333333</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Macchi Giorgio</t>
+          <t>Arco Carmelo</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1996,40 +1996,40 @@
         <v>3</v>
       </c>
       <c r="F31" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="G31" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="H31" t="n">
         <v>3</v>
       </c>
       <c r="I31" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="J31" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="K31" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="L31" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="M31" t="n">
         <v>3</v>
       </c>
       <c r="N31" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="O31" t="n">
-        <v>2.875</v>
+        <v>3.125</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Premoli Gianluca</t>
+          <t>Macchi Giorgio</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2038,19 +2038,19 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="D32" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="E32" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="F32" t="n">
         <v>2.5</v>
       </c>
       <c r="G32" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="H32" t="n">
         <v>3</v>
@@ -2059,28 +2059,28 @@
         <v>3</v>
       </c>
       <c r="J32" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="K32" t="n">
         <v>2.5</v>
       </c>
       <c r="L32" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="M32" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="N32" t="n">
         <v>2.5</v>
       </c>
       <c r="O32" t="n">
-        <v>2.75</v>
+        <v>2.875</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Colombo A lessandra</t>
+          <t>Premoli Gianluca</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2089,16 +2089,16 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D33" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="E33" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="F33" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="G33" t="n">
         <v>2.5</v>
@@ -2110,28 +2110,28 @@
         <v>3</v>
       </c>
       <c r="J33" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="K33" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="L33" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="M33" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="N33" t="n">
         <v>2.5</v>
       </c>
       <c r="O33" t="n">
-        <v>3.083333333333333</v>
+        <v>2.75</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Fernicola Alessandra</t>
+          <t>Colombo A lessandra</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2140,34 +2140,34 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D34" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="E34" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="F34" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="G34" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="H34" t="n">
         <v>3</v>
       </c>
       <c r="I34" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="J34" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="K34" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="L34" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="M34" t="n">
         <v>3</v>
@@ -2176,13 +2176,13 @@
         <v>2.5</v>
       </c>
       <c r="O34" t="n">
-        <v>2.958333333333333</v>
+        <v>3.083333333333333</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Toia Luca Luigi</t>
+          <t>Fernicola Alessandra</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2191,22 +2191,22 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="D35" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="E35" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="F35" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="G35" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="H35" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="I35" t="n">
         <v>3.5</v>
@@ -2215,7 +2215,7 @@
         <v>3</v>
       </c>
       <c r="K35" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="L35" t="n">
         <v>3</v>
@@ -2227,13 +2227,13 @@
         <v>2.5</v>
       </c>
       <c r="O35" t="n">
-        <v>2.875</v>
+        <v>2.958333333333333</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Campanello Marco</t>
+          <t>Toia Luca Luigi</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2251,7 +2251,7 @@
         <v>3</v>
       </c>
       <c r="F36" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="G36" t="n">
         <v>2.5</v>
@@ -2260,31 +2260,31 @@
         <v>2.5</v>
       </c>
       <c r="I36" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="J36" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="K36" t="n">
         <v>3</v>
       </c>
       <c r="L36" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="M36" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="N36" t="n">
         <v>2.5</v>
       </c>
       <c r="O36" t="n">
-        <v>2.75</v>
+        <v>2.875</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Milanta Mariapaola</t>
+          <t>Campanello Marco</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2293,49 +2293,49 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="D37" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="E37" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="F37" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="G37" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="H37" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="I37" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="J37" t="n">
-        <v>4</v>
+        <v>2.5</v>
       </c>
       <c r="K37" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="L37" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="M37" t="n">
-        <v>4</v>
+        <v>2.5</v>
       </c>
       <c r="N37" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="O37" t="n">
-        <v>3.541666666666667</v>
+        <v>2.75</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Calderoni Gabriele Maria</t>
+          <t>Milanta Mariapaola</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2344,49 +2344,49 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="D38" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="E38" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="F38" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="G38" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="H38" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="I38" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="J38" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="K38" t="n">
         <v>3.5</v>
       </c>
       <c r="L38" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="M38" t="n">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="N38" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="O38" t="n">
-        <v>2.916666666666667</v>
+        <v>3.541666666666667</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Ceriani Massimo</t>
+          <t>Calderoni Gabriele Maria</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2398,19 +2398,19 @@
         <v>3.5</v>
       </c>
       <c r="D39" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="E39" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="F39" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="G39" t="n">
         <v>2.5</v>
       </c>
       <c r="H39" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="I39" t="n">
         <v>3</v>
@@ -2419,7 +2419,7 @@
         <v>3.5</v>
       </c>
       <c r="K39" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="L39" t="n">
         <v>2.5</v>
@@ -2431,13 +2431,13 @@
         <v>3</v>
       </c>
       <c r="O39" t="n">
-        <v>2.833333333333333</v>
+        <v>2.916666666666667</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Valieri Andrea</t>
+          <t>Ceriani Massimo</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2446,31 +2446,31 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="D40" t="n">
         <v>2.5</v>
       </c>
       <c r="E40" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="F40" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="G40" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="H40" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="I40" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="J40" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="K40" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="L40" t="n">
         <v>2.5</v>
@@ -2479,16 +2479,16 @@
         <v>2.5</v>
       </c>
       <c r="N40" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O40" t="n">
-        <v>2.708333333333333</v>
+        <v>2.833333333333333</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Mauri Luca</t>
+          <t>Valieri Andrea</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2497,49 +2497,49 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="D41" t="n">
         <v>2.5</v>
       </c>
       <c r="E41" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F41" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G41" t="n">
+        <v>3</v>
+      </c>
+      <c r="H41" t="n">
+        <v>3</v>
+      </c>
+      <c r="I41" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J41" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K41" t="n">
+        <v>3</v>
+      </c>
+      <c r="L41" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="M41" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="N41" t="n">
         <v>2</v>
       </c>
-      <c r="F41" t="n">
-        <v>2</v>
-      </c>
-      <c r="G41" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="H41" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="I41" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="J41" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="K41" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="L41" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="M41" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="N41" t="n">
-        <v>2.5</v>
-      </c>
       <c r="O41" t="n">
-        <v>2.5</v>
+        <v>2.708333333333333</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Cercaci Alessandra</t>
+          <t>Mauri Luca</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2551,31 +2551,31 @@
         <v>2.5</v>
       </c>
       <c r="D42" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="E42" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F42" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G42" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="H42" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="I42" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="J42" t="n">
         <v>2.5</v>
       </c>
       <c r="K42" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="L42" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="M42" t="n">
         <v>2.5</v>
@@ -2584,13 +2584,13 @@
         <v>2.5</v>
       </c>
       <c r="O42" t="n">
-        <v>2.875</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Roberto Rocca</t>
+          <t>Cercaci Alessandra</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2599,10 +2599,10 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="D43" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="E43" t="n">
         <v>3</v>
@@ -2611,42 +2611,42 @@
         <v>3</v>
       </c>
       <c r="G43" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="H43" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="I43" t="n">
         <v>2.5</v>
       </c>
       <c r="J43" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="K43" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="L43" t="n">
         <v>3</v>
       </c>
       <c r="M43" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="N43" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="O43" t="n">
-        <v>2.75</v>
+        <v>2.875</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Di Sabatino Bruno</t>
+          <t>Roberto Rocca</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Dirigente Avezzano</t>
+          <t>Professional Milano</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -2656,16 +2656,16 @@
         <v>2.5</v>
       </c>
       <c r="E44" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="F44" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="G44" t="n">
         <v>2.5</v>
       </c>
       <c r="H44" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="I44" t="n">
         <v>2.5</v>
@@ -2683,16 +2683,16 @@
         <v>3</v>
       </c>
       <c r="N44" t="n">
-        <v>3.5</v>
+        <v>2</v>
       </c>
       <c r="O44" t="n">
-        <v>2.916666666666667</v>
+        <v>2.75</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Diego Gi Giampietro </t>
+          <t>Di Sabatino Bruno</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2701,16 +2701,16 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="D45" t="n">
         <v>2.5</v>
       </c>
       <c r="E45" t="n">
-        <v>2</v>
+        <v>3.5</v>
       </c>
       <c r="F45" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="G45" t="n">
         <v>2.5</v>
@@ -2719,7 +2719,7 @@
         <v>2.5</v>
       </c>
       <c r="I45" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="J45" t="n">
         <v>3</v>
@@ -2734,16 +2734,16 @@
         <v>3</v>
       </c>
       <c r="N45" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="O45" t="n">
-        <v>2.791666666666667</v>
+        <v>2.916666666666667</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Francesconi Luigia</t>
+          <t xml:space="preserve">Diego Gi Giampietro </t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2752,19 +2752,19 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="D46" t="n">
         <v>2.5</v>
       </c>
       <c r="E46" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="F46" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="G46" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="H46" t="n">
         <v>2.5</v>
@@ -2773,28 +2773,28 @@
         <v>3.5</v>
       </c>
       <c r="J46" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="K46" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="L46" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="M46" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="N46" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="O46" t="n">
-        <v>2.916666666666667</v>
+        <v>2.791666666666667</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Properzi Massimiliano</t>
+          <t>Francesconi Luigia</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2803,49 +2803,49 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D47" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="E47" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="F47" t="n">
         <v>3</v>
       </c>
       <c r="G47" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H47" t="n">
         <v>2.5</v>
       </c>
       <c r="I47" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="J47" t="n">
         <v>3.5</v>
       </c>
       <c r="K47" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="L47" t="n">
         <v>2.5</v>
       </c>
       <c r="M47" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="N47" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="O47" t="n">
-        <v>2.791666666666667</v>
+        <v>2.916666666666667</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Santangelo Maurizio</t>
+          <t>Properzi Massimiliano</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2863,10 +2863,10 @@
         <v>3.5</v>
       </c>
       <c r="F48" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="G48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H48" t="n">
         <v>2.5</v>
@@ -2875,7 +2875,7 @@
         <v>3</v>
       </c>
       <c r="J48" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="K48" t="n">
         <v>2.5</v>
@@ -2884,19 +2884,19 @@
         <v>2.5</v>
       </c>
       <c r="M48" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="N48" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="O48" t="n">
-        <v>2.875</v>
+        <v>2.791666666666667</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Santella Gianni</t>
+          <t>Santangelo Maurizio</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2905,19 +2905,19 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="D49" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="E49" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="F49" t="n">
         <v>3.5</v>
       </c>
       <c r="G49" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="H49" t="n">
         <v>2.5</v>
@@ -2929,25 +2929,25 @@
         <v>3</v>
       </c>
       <c r="K49" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="L49" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="M49" t="n">
         <v>2.5</v>
       </c>
       <c r="N49" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="O49" t="n">
-        <v>2.916666666666667</v>
+        <v>2.875</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Tartaglia Vincenzo</t>
+          <t>Santella Gianni</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2956,40 +2956,40 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="D50" t="n">
         <v>2.5</v>
       </c>
       <c r="E50" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="F50" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="G50" t="n">
         <v>2.5</v>
       </c>
       <c r="H50" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="I50" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J50" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="K50" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="L50" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="M50" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="N50" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="O50" t="n">
         <v>2.916666666666667</v>
@@ -2998,22 +2998,22 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bianchi Liberato </t>
+          <t>Tartaglia Vincenzo</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Professional Avezzano</t>
+          <t>Dirigente Avezzano</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="D51" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="E51" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="F51" t="n">
         <v>3</v>
@@ -3025,31 +3025,31 @@
         <v>3</v>
       </c>
       <c r="I51" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J51" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="K51" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="L51" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="M51" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="N51" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O51" t="n">
-        <v>2.958333333333333</v>
+        <v>2.916666666666667</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Castrigano Luca </t>
+          <t xml:space="preserve">Bianchi Liberato </t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -3058,49 +3058,49 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="D52" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="E52" t="n">
         <v>3</v>
       </c>
       <c r="F52" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="G52" t="n">
         <v>2.5</v>
       </c>
       <c r="H52" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="I52" t="n">
         <v>3</v>
       </c>
       <c r="J52" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="K52" t="n">
         <v>3</v>
       </c>
       <c r="L52" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="M52" t="n">
         <v>3</v>
       </c>
       <c r="N52" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O52" t="n">
-        <v>2.875</v>
+        <v>2.958333333333333</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">De Amicis Alvaro </t>
+          <t xml:space="preserve">Castrigano Luca </t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -3112,28 +3112,28 @@
         <v>3</v>
       </c>
       <c r="D53" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="E53" t="n">
         <v>3</v>
       </c>
       <c r="F53" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="G53" t="n">
         <v>2.5</v>
       </c>
       <c r="H53" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="I53" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="J53" t="n">
         <v>3</v>
       </c>
       <c r="K53" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="L53" t="n">
         <v>3</v>
@@ -3142,16 +3142,16 @@
         <v>3</v>
       </c>
       <c r="N53" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O53" t="n">
-        <v>2.75</v>
+        <v>2.875</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Di Giacomo Lorenzo </t>
+          <t xml:space="preserve">De Amicis Alvaro </t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3160,7 +3160,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="D54" t="n">
         <v>2.5</v>
@@ -3169,40 +3169,40 @@
         <v>3</v>
       </c>
       <c r="F54" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="G54" t="n">
-        <v>4</v>
+        <v>2.5</v>
       </c>
       <c r="H54" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="I54" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="J54" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="K54" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="L54" t="n">
         <v>3</v>
       </c>
       <c r="M54" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="N54" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O54" t="n">
-        <v>3.083333333333333</v>
+        <v>2.75</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Di Paolo Massimo</t>
+          <t xml:space="preserve">Di Giacomo Lorenzo </t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3214,46 +3214,46 @@
         <v>3.5</v>
       </c>
       <c r="D55" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="E55" t="n">
         <v>3</v>
       </c>
       <c r="F55" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="G55" t="n">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="H55" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="I55" t="n">
         <v>3</v>
       </c>
       <c r="J55" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="K55" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="L55" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M55" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="N55" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O55" t="n">
-        <v>2.75</v>
+        <v>3.083333333333333</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Volpa Alessandra </t>
+          <t>Di Paolo Massimo</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3304,7 +3304,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Amabrini Fabio</t>
+          <t xml:space="preserve">Volpa Alessandra </t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3319,43 +3319,43 @@
         <v>3</v>
       </c>
       <c r="E57" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="F57" t="n">
         <v>3</v>
       </c>
       <c r="G57" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="H57" t="n">
         <v>2.5</v>
       </c>
       <c r="I57" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="J57" t="n">
+        <v>3</v>
+      </c>
+      <c r="K57" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="L57" t="n">
         <v>2</v>
       </c>
-      <c r="K57" t="n">
+      <c r="M57" t="n">
+        <v>3</v>
+      </c>
+      <c r="N57" t="n">
         <v>2</v>
       </c>
-      <c r="L57" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="M57" t="n">
-        <v>3</v>
-      </c>
-      <c r="N57" t="n">
-        <v>2.5</v>
-      </c>
       <c r="O57" t="n">
-        <v>2.666666666666667</v>
+        <v>2.75</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Ghidelli Serge</t>
+          <t>Amabrini Fabio</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3364,13 +3364,13 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="D58" t="n">
         <v>3</v>
       </c>
       <c r="E58" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="F58" t="n">
         <v>3</v>
@@ -3379,13 +3379,13 @@
         <v>3</v>
       </c>
       <c r="H58" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="I58" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="J58" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K58" t="n">
         <v>2</v>
@@ -3400,13 +3400,13 @@
         <v>2.5</v>
       </c>
       <c r="O58" t="n">
-        <v>3.041666666666667</v>
+        <v>2.666666666666667</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Margutti Pasquale</t>
+          <t>Ghidelli Serge</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3415,13 +3415,13 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D59" t="n">
         <v>3</v>
       </c>
       <c r="E59" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="F59" t="n">
         <v>3</v>
@@ -3430,16 +3430,16 @@
         <v>3</v>
       </c>
       <c r="H59" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="I59" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="J59" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="K59" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L59" t="n">
         <v>2.5</v>
@@ -3451,13 +3451,13 @@
         <v>2.5</v>
       </c>
       <c r="O59" t="n">
-        <v>2.875</v>
+        <v>3.041666666666667</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Palma Luca</t>
+          <t>Margutti Pasquale</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3472,13 +3472,13 @@
         <v>3</v>
       </c>
       <c r="E60" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="F60" t="n">
         <v>3</v>
       </c>
       <c r="G60" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H60" t="n">
         <v>2.5</v>
@@ -3487,10 +3487,10 @@
         <v>3</v>
       </c>
       <c r="J60" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="K60" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="L60" t="n">
         <v>2.5</v>
@@ -3499,16 +3499,16 @@
         <v>3</v>
       </c>
       <c r="N60" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="O60" t="n">
-        <v>2.666666666666667</v>
+        <v>2.875</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Piccirilli Gianluca</t>
+          <t>Palma Luca</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3526,13 +3526,13 @@
         <v>3</v>
       </c>
       <c r="F61" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="G61" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H61" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="I61" t="n">
         <v>3</v>
@@ -3550,16 +3550,16 @@
         <v>3</v>
       </c>
       <c r="N61" t="n">
-        <v>3.5</v>
+        <v>2</v>
       </c>
       <c r="O61" t="n">
-        <v>2.916666666666667</v>
+        <v>2.666666666666667</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Tellone Giuliano</t>
+          <t>Piccirilli Gianluca</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3574,43 +3574,43 @@
         <v>3</v>
       </c>
       <c r="E62" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="F62" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="G62" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="H62" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="I62" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="J62" t="n">
         <v>2.5</v>
       </c>
       <c r="K62" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="L62" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="M62" t="n">
         <v>3</v>
       </c>
       <c r="N62" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="O62" t="n">
-        <v>2.75</v>
+        <v>2.916666666666667</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Zaccardelli Giuseppe</t>
+          <t>Tellone Giuliano</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3619,34 +3619,34 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D63" t="n">
         <v>3</v>
       </c>
       <c r="E63" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="F63" t="n">
         <v>3</v>
       </c>
       <c r="G63" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="H63" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="I63" t="n">
         <v>3.5</v>
       </c>
       <c r="J63" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="K63" t="n">
         <v>2</v>
       </c>
       <c r="L63" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="M63" t="n">
         <v>3</v>
@@ -3655,58 +3655,211 @@
         <v>2.5</v>
       </c>
       <c r="O63" t="n">
-        <v>3.041666666666667</v>
+        <v>2.75</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
+          <t>Zaccardelli Giuseppe</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Professional Avezzano</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>4</v>
+      </c>
+      <c r="D64" t="n">
+        <v>3</v>
+      </c>
+      <c r="E64" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F64" t="n">
+        <v>3</v>
+      </c>
+      <c r="G64" t="n">
+        <v>3</v>
+      </c>
+      <c r="H64" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I64" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J64" t="n">
+        <v>3</v>
+      </c>
+      <c r="K64" t="n">
+        <v>2</v>
+      </c>
+      <c r="L64" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="M64" t="n">
+        <v>3</v>
+      </c>
+      <c r="N64" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="O64" t="n">
+        <v>3.041666666666667</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
           <t>Lamura Sabrina</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B65" t="inlineStr">
         <is>
           <t>Professional Avezzano</t>
         </is>
       </c>
-      <c r="C64" t="n">
-        <v>3</v>
-      </c>
-      <c r="D64" t="n">
+      <c r="C65" t="n">
+        <v>3</v>
+      </c>
+      <c r="D65" t="n">
         <v>2</v>
       </c>
-      <c r="E64" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="F64" t="n">
-        <v>3</v>
-      </c>
-      <c r="G64" t="n">
-        <v>3</v>
-      </c>
-      <c r="H64" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="I64" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="J64" t="n">
-        <v>3</v>
-      </c>
-      <c r="K64" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="L64" t="n">
-        <v>3</v>
-      </c>
-      <c r="M64" t="n">
-        <v>3</v>
-      </c>
-      <c r="N64" t="n">
+      <c r="E65" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F65" t="n">
+        <v>3</v>
+      </c>
+      <c r="G65" t="n">
+        <v>3</v>
+      </c>
+      <c r="H65" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I65" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="J65" t="n">
+        <v>3</v>
+      </c>
+      <c r="K65" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="L65" t="n">
+        <v>3</v>
+      </c>
+      <c r="M65" t="n">
+        <v>3</v>
+      </c>
+      <c r="N65" t="n">
         <v>4</v>
       </c>
-      <c r="O64" t="n">
+      <c r="O65" t="n">
         <v>2.833333333333333</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Di Francesco Roberto</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Professional Avezzano</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>3</v>
+      </c>
+      <c r="D66" t="n">
+        <v>3</v>
+      </c>
+      <c r="E66" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F66" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G66" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H66" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I66" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J66" t="n">
+        <v>3</v>
+      </c>
+      <c r="K66" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="L66" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="M66" t="n">
+        <v>3</v>
+      </c>
+      <c r="N66" t="n">
+        <v>3</v>
+      </c>
+      <c r="O66" t="n">
+        <v>3.12</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Alesii Genuino</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Professional Avezzano</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D67" t="n">
+        <v>3</v>
+      </c>
+      <c r="E67" t="n">
+        <v>2</v>
+      </c>
+      <c r="F67" t="n">
+        <v>3</v>
+      </c>
+      <c r="G67" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H67" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I67" t="n">
+        <v>4</v>
+      </c>
+      <c r="J67" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K67" t="n">
+        <v>3</v>
+      </c>
+      <c r="L67" t="n">
+        <v>3</v>
+      </c>
+      <c r="M67" t="n">
+        <v>3</v>
+      </c>
+      <c r="N67" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="O67" t="n">
+        <v>2.79</v>
       </c>
     </row>
   </sheetData>
@@ -3777,13 +3930,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C2" t="n">
-        <v>3.285714285714286</v>
+        <v>3.265151515151515</v>
       </c>
       <c r="D2" t="n">
-        <v>0.4553825555391871</v>
+        <v>0.4575830901402327</v>
       </c>
       <c r="E2" t="n">
         <v>2.5</v>
@@ -3792,7 +3945,7 @@
         <v>3</v>
       </c>
       <c r="G2" t="n">
-        <v>3.5</v>
+        <v>3.25</v>
       </c>
       <c r="H2" t="n">
         <v>3.5</v>
@@ -3811,13 +3964,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C3" t="n">
         <v>2.833333333333333</v>
       </c>
       <c r="D3" t="n">
-        <v>0.3360107525161235</v>
+        <v>0.3320488070395831</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -3845,13 +3998,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C4" t="n">
-        <v>2.888888888888889</v>
+        <v>2.871212121212121</v>
       </c>
       <c r="D4" t="n">
-        <v>0.3959924694262429</v>
+        <v>0.4234528950336204</v>
       </c>
       <c r="E4" t="n">
         <v>2</v>
@@ -3879,13 +4032,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C5" t="n">
-        <v>2.952380952380953</v>
+        <v>2.954545454545455</v>
       </c>
       <c r="D5" t="n">
-        <v>0.3444758256685745</v>
+        <v>0.3478203860888849</v>
       </c>
       <c r="E5" t="n">
         <v>2</v>
@@ -3913,13 +4066,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C6" t="n">
-        <v>2.690476190476191</v>
+        <v>2.712121212121212</v>
       </c>
       <c r="D6" t="n">
-        <v>0.3527378107513292</v>
+        <v>0.3727301154022021</v>
       </c>
       <c r="E6" t="n">
         <v>2</v>
@@ -3947,13 +4100,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C7" t="n">
-        <v>2.880952380952381</v>
+        <v>2.886363636363636</v>
       </c>
       <c r="D7" t="n">
-        <v>0.3671411536835807</v>
+        <v>0.3699839346351567</v>
       </c>
       <c r="E7" t="n">
         <v>2</v>
@@ -3981,13 +4134,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C8" t="n">
-        <v>3.214285714285714</v>
+        <v>3.227272727272727</v>
       </c>
       <c r="D8" t="n">
-        <v>0.4184676897602393</v>
+        <v>0.4222815154866221</v>
       </c>
       <c r="E8" t="n">
         <v>2.5</v>
@@ -4015,13 +4168,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C9" t="n">
-        <v>3.063492063492064</v>
+        <v>3.053030303030303</v>
       </c>
       <c r="D9" t="n">
-        <v>0.4258962418324018</v>
+        <v>0.4217982372103432</v>
       </c>
       <c r="E9" t="n">
         <v>2</v>
@@ -4049,13 +4202,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C10" t="n">
-        <v>2.76984126984127</v>
+        <v>2.772727272727273</v>
       </c>
       <c r="D10" t="n">
-        <v>0.3683594495540746</v>
+        <v>0.3635489405401041</v>
       </c>
       <c r="E10" t="n">
         <v>2</v>
@@ -4083,13 +4236,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C11" t="n">
-        <v>2.793650793650793</v>
+        <v>2.787878787878788</v>
       </c>
       <c r="D11" t="n">
-        <v>0.3771168279121489</v>
+        <v>0.3727301154022021</v>
       </c>
       <c r="E11" t="n">
         <v>2</v>
@@ -4117,19 +4270,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C12" t="n">
-        <v>2.904761904761905</v>
+        <v>2.909090909090909</v>
       </c>
       <c r="D12" t="n">
-        <v>0.3220040930558188</v>
+        <v>0.3151201347116672</v>
       </c>
       <c r="E12" t="n">
         <v>2</v>
       </c>
       <c r="F12" t="n">
-        <v>2.5</v>
+        <v>2.625</v>
       </c>
       <c r="G12" t="n">
         <v>3</v>
@@ -4151,13 +4304,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C13" t="n">
-        <v>2.722222222222222</v>
+        <v>2.71969696969697</v>
       </c>
       <c r="D13" t="n">
-        <v>0.4982046620663635</v>
+        <v>0.4893385478911451</v>
       </c>
       <c r="E13" t="n">
         <v>2</v>
@@ -4309,40 +4462,40 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3.3</v>
+        <v>3.288461538461538</v>
       </c>
       <c r="C3" t="n">
-        <v>2.88</v>
+        <v>2.865384615384615</v>
       </c>
       <c r="D3" t="n">
-        <v>2.86</v>
+        <v>2.826923076923077</v>
       </c>
       <c r="E3" t="n">
-        <v>2.98</v>
+        <v>2.961538461538462</v>
       </c>
       <c r="F3" t="n">
-        <v>2.7</v>
+        <v>2.730769230769231</v>
       </c>
       <c r="G3" t="n">
-        <v>2.94</v>
+        <v>2.942307692307693</v>
       </c>
       <c r="H3" t="n">
-        <v>3.34</v>
+        <v>3.326923076923077</v>
       </c>
       <c r="I3" t="n">
-        <v>3.22</v>
+        <v>3.211538461538462</v>
       </c>
       <c r="J3" t="n">
-        <v>2.88</v>
+        <v>2.884615384615385</v>
       </c>
       <c r="K3" t="n">
-        <v>2.94</v>
+        <v>2.923076923076923</v>
       </c>
       <c r="L3" t="n">
-        <v>2.88</v>
+        <v>2.884615384615385</v>
       </c>
       <c r="M3" t="n">
-        <v>2.8</v>
+        <v>2.788461538461538</v>
       </c>
     </row>
     <row r="4">
@@ -4352,40 +4505,40 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3.321428571428572</v>
+        <v>3.25</v>
       </c>
       <c r="C4" t="n">
-        <v>2.892857142857143</v>
+        <v>2.90625</v>
       </c>
       <c r="D4" t="n">
-        <v>2.928571428571428</v>
+        <v>2.90625</v>
       </c>
       <c r="E4" t="n">
-        <v>2.892857142857143</v>
+        <v>2.9375</v>
       </c>
       <c r="F4" t="n">
-        <v>2.785714285714286</v>
+        <v>2.8125</v>
       </c>
       <c r="G4" t="n">
-        <v>2.857142857142857</v>
+        <v>2.875</v>
       </c>
       <c r="H4" t="n">
-        <v>3</v>
+        <v>3.09375</v>
       </c>
       <c r="I4" t="n">
-        <v>2.857142857142857</v>
+        <v>2.84375</v>
       </c>
       <c r="J4" t="n">
-        <v>2.5</v>
+        <v>2.53125</v>
       </c>
       <c r="K4" t="n">
-        <v>2.607142857142857</v>
+        <v>2.625</v>
       </c>
       <c r="L4" t="n">
-        <v>2.964285714285714</v>
+        <v>2.96875</v>
       </c>
       <c r="M4" t="n">
-        <v>2.642857142857143</v>
+        <v>2.65625</v>
       </c>
     </row>
     <row r="5">
@@ -4517,37 +4670,37 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1054092553389457</v>
+        <v>0.09281671450518555</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2683281572999747</v>
+        <v>0.2980446275268082</v>
       </c>
       <c r="E2" t="n">
-        <v>0.03672105410326911</v>
+        <v>0.0285596130860408</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1075828707279838</v>
+        <v>0.07106922848214556</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3031960178847316</v>
+        <v>0.2943038867849208</v>
       </c>
       <c r="H2" t="n">
-        <v>0.3083274062967545</v>
+        <v>0.2406653514695868</v>
       </c>
       <c r="I2" t="n">
-        <v>0.2583981107271907</v>
+        <v>0.284721119091158</v>
       </c>
       <c r="J2" t="n">
-        <v>0.03777415508588889</v>
+        <v>0.02101847084589152</v>
       </c>
       <c r="K2" t="n">
-        <v>-0.3085928109212778</v>
+        <v>-0.2965773573197233</v>
       </c>
       <c r="L2" t="n">
-        <v>0.1060660171779821</v>
+        <v>0.08972006315850743</v>
       </c>
       <c r="M2" t="n">
-        <v>0.08886569593131739</v>
+        <v>0.09655554741224728</v>
       </c>
     </row>
     <row r="3">
@@ -4557,40 +4710,40 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1054092553389457</v>
+        <v>0.09281671450518555</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1313198307917876</v>
+        <v>0.1458875897755232</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2438565550020666</v>
+        <v>0.2664156187101793</v>
       </c>
       <c r="F3" t="n">
-        <v>0.06804138174397707</v>
+        <v>0.04143515622105072</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1961161351381839</v>
+        <v>0.1878421764135399</v>
       </c>
       <c r="H3" t="n">
-        <v>0.08603090020146074</v>
+        <v>0.1097192038504219</v>
       </c>
       <c r="I3" t="n">
-        <v>0.1878451891913363</v>
+        <v>0.1739211160413761</v>
       </c>
       <c r="J3" t="n">
-        <v>0.1411709788979978</v>
+        <v>0.1274447165520781</v>
       </c>
       <c r="K3" t="n">
-        <v>-0.1484998492272702</v>
+        <v>-0.1346642577184154</v>
       </c>
       <c r="L3" t="n">
-        <v>0.1118033988749892</v>
+        <v>0.1102731623028519</v>
       </c>
       <c r="M3" t="n">
-        <v>-0.1124072019995688</v>
+        <v>-0.102574024744731</v>
       </c>
     </row>
     <row r="4">
@@ -4600,40 +4753,40 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.2683281572999747</v>
+        <v>0.2980446275268082</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1313198307917876</v>
+        <v>0.1458875897755232</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>0.3448652473575028</v>
+        <v>0.377460014274224</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.1058475493514314</v>
+        <v>-0.09230455544802578</v>
       </c>
       <c r="G4" t="n">
-        <v>0.1571650555971482</v>
+        <v>0.1997418321606117</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.04866642633922909</v>
+        <v>-0.07039297009212725</v>
       </c>
       <c r="I4" t="n">
-        <v>0.281592407031783</v>
+        <v>0.2972290317266504</v>
       </c>
       <c r="J4" t="n">
-        <v>0.07064393843590407</v>
+        <v>0.006813766267146065</v>
       </c>
       <c r="K4" t="n">
-        <v>0.006000300022501868</v>
+        <v>-0.005169055105089584</v>
       </c>
       <c r="L4" t="n">
-        <v>0.04216370213557821</v>
+        <v>0.02620310197755275</v>
       </c>
       <c r="M4" t="n">
-        <v>0.004541936845034168</v>
+        <v>0.04584117972040095</v>
       </c>
     </row>
     <row r="5">
@@ -4643,40 +4796,40 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.03672105410326911</v>
+        <v>0.0285596130860408</v>
       </c>
       <c r="C5" t="n">
-        <v>0.2438565550020666</v>
+        <v>0.2664156187101793</v>
       </c>
       <c r="D5" t="n">
-        <v>0.3448652473575028</v>
+        <v>0.377460014274224</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.09007268629819087</v>
+        <v>-0.0728195874927427</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.1411952721855845</v>
+        <v>-0.1005304881713207</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.1238771747338091</v>
+        <v>-0.08569971217244499</v>
       </c>
       <c r="I5" t="n">
-        <v>0.378237260718976</v>
+        <v>0.3574912634009402</v>
       </c>
       <c r="J5" t="n">
-        <v>0.07112074827585663</v>
+        <v>0.03871186426697441</v>
       </c>
       <c r="K5" t="n">
-        <v>0.04729817031952773</v>
+        <v>0.04315234814384784</v>
       </c>
       <c r="L5" t="n">
-        <v>0.1038628254749593</v>
+        <v>0.1020828435367936</v>
       </c>
       <c r="M5" t="n">
-        <v>0.03915890433862317</v>
+        <v>0.05957547354135144</v>
       </c>
     </row>
     <row r="6">
@@ -4686,40 +4839,40 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.1075828707279838</v>
+        <v>0.07106922848214556</v>
       </c>
       <c r="C6" t="n">
-        <v>0.06804138174397707</v>
+        <v>0.04143515622105072</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.1058475493514314</v>
+        <v>-0.09230455544802578</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.09007268629819087</v>
+        <v>-0.0728195874927427</v>
       </c>
       <c r="F6" t="n">
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>0.3958723802403541</v>
+        <v>0.4284925950155166</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.03512196793431376</v>
+        <v>-0.04220763444973967</v>
       </c>
       <c r="I6" t="n">
-        <v>-0.02811874169838222</v>
+        <v>-0.02372266337779877</v>
       </c>
       <c r="J6" t="n">
-        <v>-0.09162139152537169</v>
+        <v>-0.09289216833339467</v>
       </c>
       <c r="K6" t="n">
-        <v>0.02742550909624556</v>
+        <v>-0.03104026845637568</v>
       </c>
       <c r="L6" t="n">
-        <v>-0.157216660024631</v>
+        <v>-0.1280064298826935</v>
       </c>
       <c r="M6" t="n">
-        <v>0.3288786777070751</v>
+        <v>0.3099206670373668</v>
       </c>
     </row>
     <row r="7">
@@ -4729,40 +4882,40 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.3031960178847316</v>
+        <v>0.2943038867849208</v>
       </c>
       <c r="C7" t="n">
-        <v>0.1961161351381839</v>
+        <v>0.1878421764135399</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1571650555971482</v>
+        <v>0.1997418321606117</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.1411952721855845</v>
+        <v>-0.1005304881713207</v>
       </c>
       <c r="F7" t="n">
-        <v>0.3958723802403541</v>
+        <v>0.4284925950155166</v>
       </c>
       <c r="G7" t="n">
         <v>1</v>
       </c>
       <c r="H7" t="n">
-        <v>0.2212112914107082</v>
+        <v>0.1924631014664593</v>
       </c>
       <c r="I7" t="n">
-        <v>-0.002455964833900935</v>
+        <v>0.01456329666464853</v>
       </c>
       <c r="J7" t="n">
-        <v>0.1221019478288633</v>
+        <v>0.0909821637852808</v>
       </c>
       <c r="K7" t="n">
-        <v>0.1109455866630673</v>
+        <v>0.07352831512100559</v>
       </c>
       <c r="L7" t="n">
-        <v>0.2095194157233458</v>
+        <v>0.2069302762433799</v>
       </c>
       <c r="M7" t="n">
-        <v>0.2351452375237606</v>
+        <v>0.2462361749244845</v>
       </c>
     </row>
     <row r="8">
@@ -4772,40 +4925,40 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.3083274062967545</v>
+        <v>0.2406653514695868</v>
       </c>
       <c r="C8" t="n">
-        <v>0.08603090020146074</v>
+        <v>0.1097192038504219</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.04866642633922909</v>
+        <v>-0.07039297009212725</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.1238771747338091</v>
+        <v>-0.08569971217244499</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.03512196793431376</v>
+        <v>-0.04220763444973967</v>
       </c>
       <c r="G8" t="n">
-        <v>0.2212112914107082</v>
+        <v>0.1924631014664593</v>
       </c>
       <c r="H8" t="n">
         <v>1</v>
       </c>
       <c r="I8" t="n">
-        <v>0.1939258886957328</v>
+        <v>0.147227317203584</v>
       </c>
       <c r="J8" t="n">
-        <v>0.3512726896338824</v>
+        <v>0.3416333590378282</v>
       </c>
       <c r="K8" t="n">
-        <v>0.2591616786642948</v>
+        <v>0.262131624477332</v>
       </c>
       <c r="L8" t="n">
-        <v>0.1239723842102892</v>
+        <v>0.1287513590418479</v>
       </c>
       <c r="M8" t="n">
-        <v>0.1160459133258042</v>
+        <v>0.1082935125529935</v>
       </c>
     </row>
     <row r="9">
@@ -4815,40 +4968,40 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.2583981107271907</v>
+        <v>0.284721119091158</v>
       </c>
       <c r="C9" t="n">
-        <v>0.1878451891913363</v>
+        <v>0.1739211160413761</v>
       </c>
       <c r="D9" t="n">
-        <v>0.281592407031783</v>
+        <v>0.2972290317266504</v>
       </c>
       <c r="E9" t="n">
-        <v>0.378237260718976</v>
+        <v>0.3574912634009402</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.02811874169838222</v>
+        <v>-0.02372266337779877</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.002455964833900935</v>
+        <v>0.01456329666464853</v>
       </c>
       <c r="H9" t="n">
-        <v>0.1939258886957328</v>
+        <v>0.147227317203584</v>
       </c>
       <c r="I9" t="n">
         <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>0.3773756545609834</v>
+        <v>0.3557057793588415</v>
       </c>
       <c r="K9" t="n">
-        <v>0.1330989154167971</v>
+        <v>0.1215786498112198</v>
       </c>
       <c r="L9" t="n">
-        <v>-0.07280599946154354</v>
+        <v>-0.0789176796800313</v>
       </c>
       <c r="M9" t="n">
-        <v>0.06545697159084125</v>
+        <v>0.07312540616081539</v>
       </c>
     </row>
     <row r="10">
@@ -4858,40 +5011,40 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.03777415508588889</v>
+        <v>0.02101847084589152</v>
       </c>
       <c r="C10" t="n">
-        <v>0.1411709788979978</v>
+        <v>0.1274447165520781</v>
       </c>
       <c r="D10" t="n">
-        <v>0.07064393843590407</v>
+        <v>0.006813766267146065</v>
       </c>
       <c r="E10" t="n">
-        <v>0.07112074827585663</v>
+        <v>0.03871186426697441</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.09162139152537169</v>
+        <v>-0.09289216833339467</v>
       </c>
       <c r="G10" t="n">
-        <v>0.1221019478288633</v>
+        <v>0.0909821637852808</v>
       </c>
       <c r="H10" t="n">
-        <v>0.3512726896338824</v>
+        <v>0.3416333590378282</v>
       </c>
       <c r="I10" t="n">
-        <v>0.3773756545609834</v>
+        <v>0.3557057793588415</v>
       </c>
       <c r="J10" t="n">
         <v>1</v>
       </c>
       <c r="K10" t="n">
-        <v>0.2621635496140894</v>
+        <v>0.2631944769446187</v>
       </c>
       <c r="L10" t="n">
-        <v>-0.05180191265905426</v>
+        <v>-0.04883316947543471</v>
       </c>
       <c r="M10" t="n">
-        <v>0.2392501853328429</v>
+        <v>0.2201302249101322</v>
       </c>
     </row>
     <row r="11">
@@ -4901,40 +5054,40 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-0.3085928109212778</v>
+        <v>-0.2965773573197233</v>
       </c>
       <c r="C11" t="n">
-        <v>-0.1484998492272702</v>
+        <v>-0.1346642577184154</v>
       </c>
       <c r="D11" t="n">
-        <v>0.006000300022501868</v>
+        <v>-0.005169055105089584</v>
       </c>
       <c r="E11" t="n">
-        <v>0.04729817031952773</v>
+        <v>0.04315234814384784</v>
       </c>
       <c r="F11" t="n">
-        <v>0.02742550909624556</v>
+        <v>-0.03104026845637568</v>
       </c>
       <c r="G11" t="n">
-        <v>0.1109455866630673</v>
+        <v>0.07352831512100559</v>
       </c>
       <c r="H11" t="n">
-        <v>0.2591616786642948</v>
+        <v>0.262131624477332</v>
       </c>
       <c r="I11" t="n">
-        <v>0.1330989154167971</v>
+        <v>0.1215786498112198</v>
       </c>
       <c r="J11" t="n">
-        <v>0.2621635496140894</v>
+        <v>0.2631944769446187</v>
       </c>
       <c r="K11" t="n">
         <v>1</v>
       </c>
       <c r="L11" t="n">
-        <v>0.1011979451491495</v>
+        <v>0.09526059898246955</v>
       </c>
       <c r="M11" t="n">
-        <v>0.4196959498033103</v>
+        <v>0.4070504430985624</v>
       </c>
     </row>
     <row r="12">
@@ -4944,40 +5097,40 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.1060660171779821</v>
+        <v>0.08972006315850743</v>
       </c>
       <c r="C12" t="n">
-        <v>0.1118033988749892</v>
+        <v>0.1102731623028519</v>
       </c>
       <c r="D12" t="n">
-        <v>0.04216370213557821</v>
+        <v>0.02620310197755275</v>
       </c>
       <c r="E12" t="n">
-        <v>0.1038628254749593</v>
+        <v>0.1020828435367936</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.157216660024631</v>
+        <v>-0.1280064298826935</v>
       </c>
       <c r="G12" t="n">
-        <v>0.2095194157233458</v>
+        <v>0.2069302762433799</v>
       </c>
       <c r="H12" t="n">
-        <v>0.1239723842102892</v>
+        <v>0.1287513590418479</v>
       </c>
       <c r="I12" t="n">
-        <v>-0.07280599946154354</v>
+        <v>-0.0789176796800313</v>
       </c>
       <c r="J12" t="n">
-        <v>-0.05180191265905426</v>
+        <v>-0.04883316947543471</v>
       </c>
       <c r="K12" t="n">
-        <v>0.1011979451491495</v>
+        <v>0.09526059898246955</v>
       </c>
       <c r="L12" t="n">
         <v>1</v>
       </c>
       <c r="M12" t="n">
-        <v>0.08378338161052853</v>
+        <v>0.08163020465211139</v>
       </c>
     </row>
     <row r="13">
@@ -4987,37 +5140,37 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.08886569593131739</v>
+        <v>0.09655554741224728</v>
       </c>
       <c r="C13" t="n">
-        <v>-0.1124072019995688</v>
+        <v>-0.102574024744731</v>
       </c>
       <c r="D13" t="n">
-        <v>0.004541936845034168</v>
+        <v>0.04584117972040095</v>
       </c>
       <c r="E13" t="n">
-        <v>0.03915890433862317</v>
+        <v>0.05957547354135144</v>
       </c>
       <c r="F13" t="n">
-        <v>0.3288786777070751</v>
+        <v>0.3099206670373668</v>
       </c>
       <c r="G13" t="n">
-        <v>0.2351452375237606</v>
+        <v>0.2462361749244845</v>
       </c>
       <c r="H13" t="n">
-        <v>0.1160459133258042</v>
+        <v>0.1082935125529935</v>
       </c>
       <c r="I13" t="n">
-        <v>0.06545697159084125</v>
+        <v>0.07312540616081539</v>
       </c>
       <c r="J13" t="n">
-        <v>0.2392501853328429</v>
+        <v>0.2201302249101322</v>
       </c>
       <c r="K13" t="n">
-        <v>0.4196959498033103</v>
+        <v>0.4070504430985624</v>
       </c>
       <c r="L13" t="n">
-        <v>0.08378338161052853</v>
+        <v>0.08163020465211139</v>
       </c>
       <c r="M13" t="n">
         <v>1</v>

</xml_diff>